<commit_message>
Add initial Excel activity file
</commit_message>
<xml_diff>
--- a/12627539.xlsx
+++ b/12627539.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samri\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samri\Desktop\LPU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19CCDEDF-A169-4075-ADD6-9175EB5CB7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECF1B788-794D-4C0B-8049-CA5C6F41E568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="61">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1395,47 +1395,91 @@
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="13">
+        <v>46252</v>
+      </c>
+      <c r="B15" s="14">
+        <v>420</v>
+      </c>
+      <c r="C15" s="14">
+        <v>60</v>
+      </c>
+      <c r="D15" s="14">
+        <v>120</v>
+      </c>
+      <c r="E15" s="14">
+        <v>60</v>
+      </c>
+      <c r="F15" s="14">
+        <v>420</v>
+      </c>
+      <c r="G15" s="14">
+        <v>7</v>
+      </c>
+      <c r="H15" s="14">
+        <v>240</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>1320</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+        <v>120</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="A16" s="13">
+        <v>46253</v>
+      </c>
+      <c r="B16" s="14">
+        <v>330</v>
+      </c>
+      <c r="C16" s="14">
+        <v>60</v>
+      </c>
+      <c r="D16" s="14">
+        <v>180</v>
+      </c>
+      <c r="E16" s="14">
+        <v>80</v>
+      </c>
+      <c r="F16" s="14">
+        <v>420</v>
+      </c>
+      <c r="G16" s="14">
+        <v>7</v>
+      </c>
+      <c r="H16" s="14">
+        <v>120</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1190</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
+        <v>250</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Replace daily log with updated file till 25 September
</commit_message>
<xml_diff>
--- a/12627539.xlsx
+++ b/12627539.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samri\Desktop\LPU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samri\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7F75300-6B28-4317-AAAD-AEFE2A95A1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD2AA3A-9FB7-4F10-ABE8-2964DED0AD55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,15 +27,120 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="67">
+  <si>
+    <t>My Data, My Code — Daily Log</t>
+  </si>
+  <si>
+    <t>Name:</t>
+  </si>
+  <si>
+    <t>Samriddhi Choudhary</t>
+  </si>
+  <si>
+    <t>Registration No.:</t>
+  </si>
+  <si>
+    <t>Course / Section:</t>
+  </si>
+  <si>
+    <t>MCA</t>
+  </si>
+  <si>
+    <t>Month:</t>
+  </si>
+  <si>
+    <t>All durations in MINUTES. Yellow cells = enter your data. Row 6 is a sample — overwrite it. Rows 2-3: fill your details.</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Sleep (min)</t>
+  </si>
+  <si>
+    <t>Fitness (min)</t>
+  </si>
+  <si>
+    <t>Study (min)</t>
+  </si>
+  <si>
+    <t>Coding (min)</t>
+  </si>
+  <si>
+    <t>Class (min)</t>
+  </si>
+  <si>
+    <t>Classes Attended</t>
+  </si>
+  <si>
+    <t>Other Activities (min)</t>
+  </si>
+  <si>
+    <t>Total Tracked (min)</t>
+  </si>
+  <si>
+    <t>Free/Unaccounted (min)</t>
+  </si>
+  <si>
+    <t>Day's Feeling</t>
+  </si>
+  <si>
+    <t>Satisfaction Level</t>
+  </si>
+  <si>
+    <t>Energy Level</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Satisfied</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Example row — replace with your own data. Felt a bit tired after evening class.</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Worked on assignments and revised class topics.</t>
+  </si>
+  <si>
+    <t>Focused on studies and completed daily tasks.</t>
+  </si>
+  <si>
+    <t>Completed classes and spent time on coding practice.</t>
+  </si>
+  <si>
+    <t>Productive day with a good balance of study and activities.</t>
+  </si>
+  <si>
+    <t>Regular day with classes and study.</t>
+  </si>
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -118,109 +223,16 @@
     <t xml:space="preserve">   Notes               - short free-text note (exams, illness, travel, anything explaining an unusual day)</t>
   </si>
   <si>
+    <t>5. GOOD PRACTICE</t>
+  </si>
+  <si>
     <t xml:space="preserve">   Fill this in at the same time every day (e.g. before bed) so entries stay accurate.</t>
   </si>
   <si>
     <t xml:space="preserve">   Keep every duration in minutes — do not mix hours and minutes in the same column.</t>
   </si>
   <si>
-    <t>My Data, My Code — Daily Log</t>
-  </si>
-  <si>
-    <t>Name:</t>
-  </si>
-  <si>
-    <t>Registration No.:</t>
-  </si>
-  <si>
-    <t>Course / Section:</t>
-  </si>
-  <si>
-    <t>Month:</t>
-  </si>
-  <si>
-    <t>All durations in MINUTES. Yellow cells = enter your data. Row 6 is a sample — overwrite it. Rows 2-3: fill your details.</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Sleep (min)</t>
-  </si>
-  <si>
-    <t>Fitness (min)</t>
-  </si>
-  <si>
-    <t>Study (min)</t>
-  </si>
-  <si>
-    <t>Coding (min)</t>
-  </si>
-  <si>
-    <t>Class (min)</t>
-  </si>
-  <si>
-    <t>Classes Attended</t>
-  </si>
-  <si>
-    <t>Other Activities (min)</t>
-  </si>
-  <si>
-    <t>Total Tracked (min)</t>
-  </si>
-  <si>
-    <t>Free/Unaccounted (min)</t>
-  </si>
-  <si>
-    <t>Day's Feeling</t>
-  </si>
-  <si>
-    <t>Satisfaction Level</t>
-  </si>
-  <si>
-    <t>Energy Level</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Good</t>
-  </si>
-  <si>
-    <t>Satisfied</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Example row — replace with your own data. Felt a bit tired after evening class.</t>
-  </si>
-  <si>
-    <t>5. GOOD PRACTICE</t>
-  </si>
-  <si>
-    <t>Samriddhi Choudhary</t>
-  </si>
-  <si>
-    <t>MCA</t>
-  </si>
-  <si>
-    <t>August</t>
-  </si>
-  <si>
-    <t>Neutral</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Very Satisfied</t>
-  </si>
-  <si>
-    <t>Unsatisfied</t>
-  </si>
-  <si>
-    <t>High</t>
+    <t>September</t>
   </si>
 </sst>
 </file>
@@ -332,7 +344,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -355,11 +367,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -400,9 +436,12 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -686,19 +725,19 @@
     <col min="1" max="1" width="105" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="22.8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" ht="22.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="16.8" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>1</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
@@ -706,12 +745,12 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>3</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
@@ -719,22 +758,22 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>5</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
@@ -742,17 +781,17 @@
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>9</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
@@ -760,77 +799,77 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>16</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>18</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>26</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
@@ -838,17 +877,17 @@
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
@@ -886,120 +925,120 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>54</v>
+        <v>1</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>2</v>
       </c>
       <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
+      <c r="D2" s="19"/>
       <c r="E2" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="20">
+        <v>3</v>
+      </c>
+      <c r="F2" s="18">
         <v>12627539</v>
       </c>
-      <c r="G2" s="20"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>55</v>
+        <v>4</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>5</v>
       </c>
       <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="D3" s="19"/>
       <c r="E3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="G3" s="20"/>
+        <v>6</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="19"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-    </row>
-    <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+    </row>
+    <row r="5" spans="1:14" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>46223</v>
       </c>
@@ -1033,19 +1072,19 @@
         <v>555</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
         <v>46244</v>
       </c>
@@ -1079,17 +1118,19 @@
         <v>955</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N7" s="17"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
         <v>46245</v>
       </c>
@@ -1123,15 +1164,17 @@
         <v>445</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N8" s="17"/>
+        <v>24</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
@@ -1167,17 +1210,19 @@
         <v>530</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N9" s="17"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
         <v>46247</v>
       </c>
@@ -1211,17 +1256,19 @@
         <v>610</v>
       </c>
       <c r="K10" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N10" s="17"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
         <v>46248</v>
       </c>
@@ -1255,17 +1302,19 @@
         <v>500</v>
       </c>
       <c r="K11" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N11" s="17"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
         <v>46249</v>
       </c>
@@ -1299,17 +1348,19 @@
         <v>360</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N12" s="17"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>46250</v>
       </c>
@@ -1343,17 +1394,19 @@
         <v>570</v>
       </c>
       <c r="K13" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N13" s="17"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
         <v>46251</v>
       </c>
@@ -1387,17 +1440,19 @@
         <v>560</v>
       </c>
       <c r="K14" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L14" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N14" s="17"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="13">
         <v>46252</v>
       </c>
@@ -1431,15 +1486,17 @@
         <v>120</v>
       </c>
       <c r="K15" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M15" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N15" s="17"/>
+        <v>24</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
@@ -1475,17 +1532,19 @@
         <v>250</v>
       </c>
       <c r="K16" s="16" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="L16" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M16" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N16" s="17"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
         <v>46254</v>
       </c>
@@ -1519,15 +1578,17 @@
         <v>180</v>
       </c>
       <c r="K17" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N17" s="17"/>
+        <v>24</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="13">
@@ -1563,17 +1624,19 @@
         <v>300</v>
       </c>
       <c r="K18" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="N18" s="17"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="13">
         <v>46256</v>
       </c>
@@ -1607,15 +1670,17 @@
         <v>420</v>
       </c>
       <c r="K19" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L19" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="N19" s="17"/>
+        <v>30</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="13">
@@ -1651,741 +1716,1535 @@
         <v>130</v>
       </c>
       <c r="K20" s="16" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="L20" s="16" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="N20" s="17"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+        <v>24</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B21" s="14">
+        <v>330</v>
+      </c>
+      <c r="C21" s="14">
+        <v>30</v>
+      </c>
+      <c r="D21" s="14">
+        <v>210</v>
+      </c>
+      <c r="E21" s="14">
+        <v>60</v>
+      </c>
+      <c r="F21" s="14">
+        <v>300</v>
+      </c>
+      <c r="G21" s="14">
+        <v>5</v>
+      </c>
+      <c r="H21" s="14">
+        <v>45</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>975</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+        <v>465</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B22" s="14">
+        <v>480</v>
+      </c>
+      <c r="C22" s="14">
+        <v>30</v>
+      </c>
+      <c r="D22" s="14">
+        <v>60</v>
+      </c>
+      <c r="E22" s="14">
+        <v>30</v>
+      </c>
+      <c r="F22" s="14">
+        <v>300</v>
+      </c>
+      <c r="G22" s="14">
+        <v>5</v>
+      </c>
+      <c r="H22" s="14">
+        <v>45</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>945</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+        <v>495</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B23" s="14">
+        <v>480</v>
+      </c>
+      <c r="C23" s="14">
+        <v>45</v>
+      </c>
+      <c r="D23" s="14">
+        <v>150</v>
+      </c>
+      <c r="E23" s="14">
+        <v>90</v>
+      </c>
+      <c r="F23" s="14">
+        <v>360</v>
+      </c>
+      <c r="G23" s="14">
+        <v>6</v>
+      </c>
+      <c r="H23" s="14">
+        <v>180</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1305</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+        <v>135</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B24" s="14">
+        <v>420</v>
+      </c>
+      <c r="C24" s="14">
+        <v>45</v>
+      </c>
+      <c r="D24" s="14">
+        <v>90</v>
+      </c>
+      <c r="E24" s="14">
+        <v>60</v>
+      </c>
+      <c r="F24" s="14">
+        <v>300</v>
+      </c>
+      <c r="G24" s="14">
+        <v>5</v>
+      </c>
+      <c r="H24" s="14">
+        <v>30</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>945</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+        <v>495</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N24" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B25" s="14">
+        <v>420</v>
+      </c>
+      <c r="C25" s="14">
+        <v>30</v>
+      </c>
+      <c r="D25" s="14">
+        <v>210</v>
+      </c>
+      <c r="E25" s="14">
+        <v>75</v>
+      </c>
+      <c r="F25" s="14">
+        <v>420</v>
+      </c>
+      <c r="G25" s="14">
+        <v>7</v>
+      </c>
+      <c r="H25" s="14">
+        <v>30</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>1185</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="17"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+        <v>255</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <v>46263</v>
+      </c>
+      <c r="B26" s="14">
+        <v>450</v>
+      </c>
+      <c r="C26" s="14">
+        <v>45</v>
+      </c>
+      <c r="D26" s="14">
+        <v>60</v>
+      </c>
+      <c r="E26" s="14">
+        <v>30</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0</v>
+      </c>
+      <c r="G26" s="14">
+        <v>0</v>
+      </c>
+      <c r="H26" s="14">
+        <v>150</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>735</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="17"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+        <v>705</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <v>46264</v>
+      </c>
+      <c r="B27" s="14">
+        <v>330</v>
+      </c>
+      <c r="C27" s="14">
+        <v>90</v>
+      </c>
+      <c r="D27" s="14">
+        <v>120</v>
+      </c>
+      <c r="E27" s="14">
+        <v>75</v>
+      </c>
+      <c r="F27" s="14">
+        <v>0</v>
+      </c>
+      <c r="G27" s="14">
+        <v>0</v>
+      </c>
+      <c r="H27" s="14">
+        <v>150</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>765</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="17"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+        <v>675</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B28" s="14">
+        <v>390</v>
+      </c>
+      <c r="C28" s="14">
+        <v>90</v>
+      </c>
+      <c r="D28" s="14">
+        <v>120</v>
+      </c>
+      <c r="E28" s="14">
+        <v>120</v>
+      </c>
+      <c r="F28" s="14">
+        <v>420</v>
+      </c>
+      <c r="G28" s="14">
+        <v>7</v>
+      </c>
+      <c r="H28" s="14">
+        <v>150</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1290</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+        <v>150</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B29" s="14">
+        <v>510</v>
+      </c>
+      <c r="C29" s="14">
+        <v>60</v>
+      </c>
+      <c r="D29" s="14">
+        <v>120</v>
+      </c>
+      <c r="E29" s="14">
+        <v>120</v>
+      </c>
+      <c r="F29" s="14">
+        <v>420</v>
+      </c>
+      <c r="G29" s="14">
+        <v>7</v>
+      </c>
+      <c r="H29" s="14">
+        <v>120</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>1350</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="17"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+        <v>90</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N29" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B30" s="14">
+        <v>300</v>
+      </c>
+      <c r="C30" s="14">
+        <v>60</v>
+      </c>
+      <c r="D30" s="14">
+        <v>150</v>
+      </c>
+      <c r="E30" s="14">
+        <v>60</v>
+      </c>
+      <c r="F30" s="14">
+        <v>300</v>
+      </c>
+      <c r="G30" s="14">
+        <v>5</v>
+      </c>
+      <c r="H30" s="14">
+        <v>45</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>915</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="17"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+        <v>525</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N30" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B31" s="14">
+        <v>480</v>
+      </c>
+      <c r="C31" s="14">
+        <v>90</v>
+      </c>
+      <c r="D31" s="14">
+        <v>150</v>
+      </c>
+      <c r="E31" s="14">
+        <v>45</v>
+      </c>
+      <c r="F31" s="14">
+        <v>360</v>
+      </c>
+      <c r="G31" s="14">
+        <v>6</v>
+      </c>
+      <c r="H31" s="14">
+        <v>45</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>1170</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="17"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+        <v>270</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N31" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B32" s="14">
+        <v>480</v>
+      </c>
+      <c r="C32" s="14">
+        <v>60</v>
+      </c>
+      <c r="D32" s="14">
+        <v>90</v>
+      </c>
+      <c r="E32" s="14">
+        <v>45</v>
+      </c>
+      <c r="F32" s="14">
+        <v>420</v>
+      </c>
+      <c r="G32" s="14">
+        <v>7</v>
+      </c>
+      <c r="H32" s="14">
+        <v>90</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>1185</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="17"/>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+        <v>255</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B33" s="14">
+        <v>360</v>
+      </c>
+      <c r="C33" s="14">
+        <v>90</v>
+      </c>
+      <c r="D33" s="14">
+        <v>180</v>
+      </c>
+      <c r="E33" s="14">
+        <v>30</v>
+      </c>
+      <c r="F33" s="14">
+        <v>0</v>
+      </c>
+      <c r="G33" s="14">
+        <v>0</v>
+      </c>
+      <c r="H33" s="14">
+        <v>90</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+        <v>690</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A34" s="13">
+        <v>46271</v>
+      </c>
+      <c r="B34" s="14">
+        <v>300</v>
+      </c>
+      <c r="C34" s="14">
+        <v>30</v>
+      </c>
+      <c r="D34" s="14">
+        <v>180</v>
+      </c>
+      <c r="E34" s="14">
+        <v>60</v>
+      </c>
+      <c r="F34" s="14">
+        <v>0</v>
+      </c>
+      <c r="G34" s="14">
+        <v>0</v>
+      </c>
+      <c r="H34" s="14">
+        <v>180</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
-    </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+        <v>690</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="13">
+        <v>46272</v>
+      </c>
+      <c r="B35" s="14">
+        <v>360</v>
+      </c>
+      <c r="C35" s="14">
+        <v>60</v>
+      </c>
+      <c r="D35" s="14">
+        <v>60</v>
+      </c>
+      <c r="E35" s="14">
+        <v>120</v>
+      </c>
+      <c r="F35" s="14">
+        <v>420</v>
+      </c>
+      <c r="G35" s="14">
+        <v>7</v>
+      </c>
+      <c r="H35" s="14">
+        <v>60</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+        <v>360</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="13">
+        <v>46273</v>
+      </c>
+      <c r="B36" s="14">
+        <v>390</v>
+      </c>
+      <c r="C36" s="14">
+        <v>45</v>
+      </c>
+      <c r="D36" s="14">
+        <v>120</v>
+      </c>
+      <c r="E36" s="14">
+        <v>45</v>
+      </c>
+      <c r="F36" s="14">
+        <v>420</v>
+      </c>
+      <c r="G36" s="14">
+        <v>7</v>
+      </c>
+      <c r="H36" s="14">
+        <v>180</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
-      <c r="N36" s="17"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+        <v>240</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N36" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="13">
+        <v>46274</v>
+      </c>
+      <c r="B37" s="14">
+        <v>300</v>
+      </c>
+      <c r="C37" s="14">
+        <v>30</v>
+      </c>
+      <c r="D37" s="14">
+        <v>120</v>
+      </c>
+      <c r="E37" s="14">
+        <v>60</v>
+      </c>
+      <c r="F37" s="14">
+        <v>300</v>
+      </c>
+      <c r="G37" s="14">
+        <v>5</v>
+      </c>
+      <c r="H37" s="14">
+        <v>30</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B38" s="14">
+        <v>330</v>
+      </c>
+      <c r="C38" s="14">
+        <v>75</v>
+      </c>
+      <c r="D38" s="14">
+        <v>90</v>
+      </c>
+      <c r="E38" s="14">
+        <v>45</v>
+      </c>
+      <c r="F38" s="14">
+        <v>420</v>
+      </c>
+      <c r="G38" s="14">
+        <v>7</v>
+      </c>
+      <c r="H38" s="14">
+        <v>90</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+        <v>390</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B39" s="14">
+        <v>480</v>
+      </c>
+      <c r="C39" s="14">
+        <v>45</v>
+      </c>
+      <c r="D39" s="14">
+        <v>180</v>
+      </c>
+      <c r="E39" s="14">
+        <v>120</v>
+      </c>
+      <c r="F39" s="14">
+        <v>420</v>
+      </c>
+      <c r="G39" s="14">
+        <v>7</v>
+      </c>
+      <c r="H39" s="14">
+        <v>45</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>1290</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+        <v>150</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A40" s="13">
+        <v>46277</v>
+      </c>
+      <c r="B40" s="14">
+        <v>510</v>
+      </c>
+      <c r="C40" s="14">
+        <v>30</v>
+      </c>
+      <c r="D40" s="14">
+        <v>90</v>
+      </c>
+      <c r="E40" s="14">
+        <v>45</v>
+      </c>
+      <c r="F40" s="14">
+        <v>0</v>
+      </c>
+      <c r="G40" s="14">
+        <v>0</v>
+      </c>
+      <c r="H40" s="14">
+        <v>30</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>705</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+        <v>735</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="13">
+        <v>46278</v>
+      </c>
+      <c r="B41" s="14">
+        <v>390</v>
+      </c>
+      <c r="C41" s="14">
+        <v>30</v>
+      </c>
+      <c r="D41" s="14">
+        <v>60</v>
+      </c>
+      <c r="E41" s="14">
+        <v>120</v>
+      </c>
+      <c r="F41" s="14">
+        <v>0</v>
+      </c>
+      <c r="G41" s="14">
+        <v>0</v>
+      </c>
+      <c r="H41" s="14">
+        <v>150</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
-    </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+        <v>690</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="13">
+        <v>46279</v>
+      </c>
+      <c r="B42" s="14">
+        <v>450</v>
+      </c>
+      <c r="C42" s="14">
+        <v>30</v>
+      </c>
+      <c r="D42" s="14">
+        <v>180</v>
+      </c>
+      <c r="E42" s="14">
+        <v>45</v>
+      </c>
+      <c r="F42" s="14">
+        <v>360</v>
+      </c>
+      <c r="G42" s="14">
+        <v>6</v>
+      </c>
+      <c r="H42" s="14">
+        <v>150</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>1215</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
-      <c r="N42" s="17"/>
-    </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+        <v>225</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N42" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A43" s="13">
+        <v>46280</v>
+      </c>
+      <c r="B43" s="14">
+        <v>510</v>
+      </c>
+      <c r="C43" s="14">
+        <v>45</v>
+      </c>
+      <c r="D43" s="14">
+        <v>150</v>
+      </c>
+      <c r="E43" s="14">
+        <v>75</v>
+      </c>
+      <c r="F43" s="14">
+        <v>300</v>
+      </c>
+      <c r="G43" s="14">
+        <v>5</v>
+      </c>
+      <c r="H43" s="14">
+        <v>30</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>1110</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
-      <c r="N43" s="17"/>
-    </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+        <v>330</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="N43" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="13">
+        <v>46281</v>
+      </c>
+      <c r="B44" s="14">
+        <v>480</v>
+      </c>
+      <c r="C44" s="14">
+        <v>60</v>
+      </c>
+      <c r="D44" s="14">
+        <v>210</v>
+      </c>
+      <c r="E44" s="14">
+        <v>30</v>
+      </c>
+      <c r="F44" s="14">
+        <v>420</v>
+      </c>
+      <c r="G44" s="14">
+        <v>7</v>
+      </c>
+      <c r="H44" s="14">
+        <v>150</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>1350</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
-      <c r="N44" s="17"/>
-    </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+        <v>90</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N44" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="13">
+        <v>46282</v>
+      </c>
+      <c r="B45" s="14">
+        <v>330</v>
+      </c>
+      <c r="C45" s="14">
+        <v>45</v>
+      </c>
+      <c r="D45" s="14">
+        <v>90</v>
+      </c>
+      <c r="E45" s="14">
+        <v>45</v>
+      </c>
+      <c r="F45" s="14">
+        <v>420</v>
+      </c>
+      <c r="G45" s="14">
+        <v>7</v>
+      </c>
+      <c r="H45" s="14">
+        <v>90</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="17"/>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+        <v>420</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N45" s="17" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="13">
+        <v>46283</v>
+      </c>
+      <c r="B46" s="14">
+        <v>510</v>
+      </c>
+      <c r="C46" s="14">
+        <v>45</v>
+      </c>
+      <c r="D46" s="14">
+        <v>60</v>
+      </c>
+      <c r="E46" s="14">
+        <v>75</v>
+      </c>
+      <c r="F46" s="14">
+        <v>420</v>
+      </c>
+      <c r="G46" s="14">
+        <v>7</v>
+      </c>
+      <c r="H46" s="14">
+        <v>30</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
-      <c r="N46" s="17"/>
-    </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A47" s="13"/>
-      <c r="B47" s="14"/>
-      <c r="C47" s="14"/>
-      <c r="D47" s="14"/>
-      <c r="E47" s="14"/>
-      <c r="F47" s="14"/>
-      <c r="G47" s="14"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="15" t="str">
+        <v>300</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N46" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A47" s="13">
+        <v>46284</v>
+      </c>
+      <c r="B47" s="14">
+        <v>360</v>
+      </c>
+      <c r="C47" s="14">
+        <v>90</v>
+      </c>
+      <c r="D47" s="14">
+        <v>150</v>
+      </c>
+      <c r="E47" s="14">
+        <v>75</v>
+      </c>
+      <c r="F47" s="14">
+        <v>0</v>
+      </c>
+      <c r="G47" s="14">
+        <v>0</v>
+      </c>
+      <c r="H47" s="14">
+        <v>45</v>
+      </c>
+      <c r="I47" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J47" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="J47" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="16"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="17"/>
-    </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="K47" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L47" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M47" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N47" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A48" s="13">
+        <v>46285</v>
+      </c>
+      <c r="B48" s="14">
+        <v>300</v>
+      </c>
+      <c r="C48" s="14">
+        <v>90</v>
+      </c>
+      <c r="D48" s="14">
+        <v>120</v>
+      </c>
+      <c r="E48" s="14">
+        <v>75</v>
+      </c>
+      <c r="F48" s="14">
+        <v>0</v>
+      </c>
+      <c r="G48" s="14">
+        <v>0</v>
+      </c>
+      <c r="H48" s="14">
+        <v>60</v>
+      </c>
+      <c r="I48" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J48" s="15" t="str">
+        <v>645</v>
+      </c>
+      <c r="J48" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K48" s="16"/>
-      <c r="L48" s="16"/>
-      <c r="M48" s="16"/>
-      <c r="N48" s="17"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="13"/>
-      <c r="B49" s="14"/>
-      <c r="C49" s="14"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="14"/>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="15" t="str">
+        <v>795</v>
+      </c>
+      <c r="K48" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L48" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="M48" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N48" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="13">
+        <v>46286</v>
+      </c>
+      <c r="B49" s="14">
+        <v>420</v>
+      </c>
+      <c r="C49" s="14">
+        <v>45</v>
+      </c>
+      <c r="D49" s="14">
+        <v>60</v>
+      </c>
+      <c r="E49" s="14">
+        <v>90</v>
+      </c>
+      <c r="F49" s="14">
+        <v>420</v>
+      </c>
+      <c r="G49" s="14">
+        <v>7</v>
+      </c>
+      <c r="H49" s="14">
+        <v>120</v>
+      </c>
+      <c r="I49" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J49" s="15" t="str">
+        <v>1155</v>
+      </c>
+      <c r="J49" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="16"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="17"/>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="13"/>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+        <v>285</v>
+      </c>
+      <c r="K49" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L49" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M49" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N49" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A50" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B50" s="14">
+        <v>510</v>
+      </c>
+      <c r="C50" s="14">
+        <v>75</v>
+      </c>
+      <c r="D50" s="14">
+        <v>180</v>
+      </c>
+      <c r="E50" s="14">
+        <v>45</v>
+      </c>
+      <c r="F50" s="14">
+        <v>300</v>
+      </c>
+      <c r="G50" s="14">
+        <v>5</v>
+      </c>
+      <c r="H50" s="14">
+        <v>120</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>1230</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
-    </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+        <v>210</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N50" s="17" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A51" s="13">
+        <v>46288</v>
+      </c>
+      <c r="B51" s="14">
+        <v>330</v>
+      </c>
+      <c r="C51" s="14">
+        <v>90</v>
+      </c>
+      <c r="D51" s="14">
+        <v>90</v>
+      </c>
+      <c r="E51" s="14">
+        <v>75</v>
+      </c>
+      <c r="F51" s="14">
+        <v>300</v>
+      </c>
+      <c r="G51" s="14">
+        <v>5</v>
+      </c>
+      <c r="H51" s="14">
+        <v>120</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>1005</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
-    </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+        <v>435</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N51" s="17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A52" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B52" s="14">
+        <v>450</v>
+      </c>
+      <c r="C52" s="14">
+        <v>60</v>
+      </c>
+      <c r="D52" s="14">
+        <v>90</v>
+      </c>
+      <c r="E52" s="14">
+        <v>120</v>
+      </c>
+      <c r="F52" s="14">
+        <v>420</v>
+      </c>
+      <c r="G52" s="14">
+        <v>7</v>
+      </c>
+      <c r="H52" s="14">
+        <v>60</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
-    </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14"/>
-      <c r="C53" s="14"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="14"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="15" t="str">
+        <v>240</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A53" s="13">
+        <v>46290</v>
+      </c>
+      <c r="B53" s="14">
+        <v>420</v>
+      </c>
+      <c r="C53" s="14">
+        <v>60</v>
+      </c>
+      <c r="D53" s="14">
+        <v>120</v>
+      </c>
+      <c r="E53" s="14">
+        <v>30</v>
+      </c>
+      <c r="F53" s="14">
+        <v>300</v>
+      </c>
+      <c r="G53" s="14">
+        <v>5</v>
+      </c>
+      <c r="H53" s="14">
+        <v>90</v>
+      </c>
+      <c r="I53" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J53" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="16"/>
-      <c r="L53" s="16"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="17"/>
+        <v>420</v>
+      </c>
+      <c r="K53" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="L53" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M53" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N53" s="17" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54" s="13"/>
@@ -9789,11 +10648,11 @@
       <c r="G390" s="14"/>
       <c r="H390" s="14"/>
       <c r="I390" s="15" t="str">
-        <f t="shared" ref="I390:I401" si="12">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
+        <f t="shared" ref="I390:I453" si="12">IF(SUM(B390:F390,H390)=0,"",SUM(B390:F390,H390))</f>
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J401" si="13">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J453" si="13">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>
@@ -10045,12 +10904,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A4:N4"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F3:G3"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <conditionalFormatting sqref="J6:J401">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">

</xml_diff>